<commit_message>
chore(data-release): publish site data 2026-10-23 03:56:11 UTC
</commit_message>
<xml_diff>
--- a/countries/fi/2026-2029.xlsx
+++ b/countries/fi/2026-2029.xlsx
@@ -53608,13 +53608,13 @@
         </is>
       </c>
       <c r="N369" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="O369" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="R369" t="n">
-        <v>1.245166419604896</v>
+        <v>1.316318786439462</v>
       </c>
       <c r="U369" t="inlineStr">
         <is>
@@ -54328,13 +54328,13 @@
         </is>
       </c>
       <c r="N374" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O374" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="R374" t="n">
-        <v>1.867749629407345</v>
+        <v>1.849961537698703</v>
       </c>
       <c r="U374" t="inlineStr">
         <is>
@@ -56488,13 +56488,13 @@
         </is>
       </c>
       <c r="N389" t="n">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="O389" t="n">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="R389" t="n">
-        <v>3.486465974893709</v>
+        <v>3.522042158310993</v>
       </c>
       <c r="U389" t="inlineStr">
         <is>
@@ -60376,13 +60376,13 @@
         </is>
       </c>
       <c r="N416" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="O416" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="R416" t="n">
-        <v>0.6225832098024481</v>
+        <v>0.6937355766370136</v>
       </c>
       <c r="U416" t="inlineStr">
         <is>
@@ -61096,13 +61096,13 @@
         </is>
       </c>
       <c r="N421" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O421" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="R421" t="n">
-        <v>1.42304733669131</v>
+        <v>1.405259244982669</v>
       </c>
       <c r="U421" t="inlineStr">
         <is>
@@ -61672,13 +61672,13 @@
         </is>
       </c>
       <c r="N425" t="n">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="O425" t="n">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="R425" t="n">
-        <v>1.209590236187614</v>
+        <v>1.476411611817234</v>
       </c>
       <c r="U425" t="inlineStr">
         <is>
@@ -62104,13 +62104,13 @@
         </is>
       </c>
       <c r="N428" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="O428" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="R428" t="n">
-        <v>0.569218934676524</v>
+        <v>0.6403713015110895</v>
       </c>
       <c r="U428" t="inlineStr">
         <is>
@@ -62824,13 +62824,13 @@
         </is>
       </c>
       <c r="N433" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O433" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R433" t="n">
-        <v>0.142304733669131</v>
+        <v>0.1600928253777724</v>
       </c>
       <c r="U433" t="inlineStr">
         <is>
@@ -62968,13 +62968,13 @@
         </is>
       </c>
       <c r="N434" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="O434" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="R434" t="n">
-        <v>0.5158546595505998</v>
+        <v>0.6403713015110895</v>
       </c>
       <c r="U434" t="inlineStr">
         <is>
@@ -63256,13 +63256,13 @@
         </is>
       </c>
       <c r="N436" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="O436" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="R436" t="n">
-        <v>1.796597262572779</v>
+        <v>1.903325812824627</v>
       </c>
       <c r="U436" t="inlineStr">
         <is>
@@ -63688,13 +63688,13 @@
         </is>
       </c>
       <c r="N439" t="n">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="O439" t="n">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="R439" t="n">
-        <v>2.116782913328324</v>
+        <v>2.45475665579251</v>
       </c>
       <c r="U439" t="inlineStr">
         <is>
@@ -64696,13 +64696,13 @@
         </is>
       </c>
       <c r="N446" t="n">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="O446" t="n">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="R446" t="n">
-        <v>1.832173445990062</v>
+        <v>2.045630546493758</v>
       </c>
       <c r="U446" t="inlineStr">
         <is>
@@ -64840,13 +64840,13 @@
         </is>
       </c>
       <c r="N447" t="n">
-        <v>493</v>
+        <v>562</v>
       </c>
       <c r="O447" t="n">
-        <v>493</v>
+        <v>562</v>
       </c>
       <c r="R447" t="n">
-        <v>8.769529212360197</v>
+        <v>9.996907540256453</v>
       </c>
       <c r="U447" t="inlineStr">
         <is>
@@ -64984,13 +64984,13 @@
         </is>
       </c>
       <c r="N448" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="O448" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="R448" t="n">
-        <v>0.4447022927160344</v>
+        <v>0.569218934676524</v>
       </c>
       <c r="U448" t="inlineStr">
         <is>
@@ -65128,13 +65128,13 @@
         </is>
       </c>
       <c r="N449" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="O449" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="R449" t="n">
-        <v>0.2668213756296206</v>
+        <v>0.3379737424641861</v>
       </c>
       <c r="U449" t="inlineStr">
         <is>
@@ -65272,13 +65272,13 @@
         </is>
       </c>
       <c r="N450" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O450" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R450" t="n">
-        <v>0.03557618341728275</v>
+        <v>0.05336427512592412</v>
       </c>
       <c r="U450" t="inlineStr">
         <is>
@@ -65416,13 +65416,13 @@
         </is>
       </c>
       <c r="N451" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="O451" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="R451" t="n">
-        <v>0.7115236683456551</v>
+        <v>0.8182522185975032</v>
       </c>
       <c r="U451" t="inlineStr">
         <is>
@@ -65704,13 +65704,13 @@
         </is>
       </c>
       <c r="N453" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="O453" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="R453" t="n">
-        <v>0.426914201007393</v>
+        <v>0.4980665678419585</v>
       </c>
       <c r="U453" t="inlineStr">
         <is>
@@ -65848,13 +65848,13 @@
         </is>
       </c>
       <c r="N454" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O454" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R454" t="n">
-        <v>0.07115236683456549</v>
+        <v>0.1067285502518482</v>
       </c>
       <c r="U454" t="inlineStr">
         <is>
@@ -66136,13 +66136,13 @@
         </is>
       </c>
       <c r="N456" t="n">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="O456" t="n">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="R456" t="n">
-        <v>2.810518489965337</v>
+        <v>3.148492232429523</v>
       </c>
       <c r="U456" t="inlineStr">
         <is>
@@ -66424,13 +66424,13 @@
         </is>
       </c>
       <c r="N458" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="O458" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="R458" t="n">
-        <v>0.5336427512592412</v>
+        <v>0.569218934676524</v>
       </c>
       <c r="U458" t="inlineStr">
         <is>
@@ -67000,13 +67000,13 @@
         </is>
       </c>
       <c r="N462" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O462" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R462" t="n">
-        <v>0.07115236683456549</v>
+        <v>0.08894045854320688</v>
       </c>
       <c r="U462" t="inlineStr">
         <is>
@@ -67144,13 +67144,13 @@
         </is>
       </c>
       <c r="N463" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O463" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R463" t="n">
-        <v>0.01778809170864137</v>
+        <v>0.03557618341728275</v>
       </c>
       <c r="U463" t="inlineStr">
         <is>
@@ -67288,13 +67288,13 @@
         </is>
       </c>
       <c r="N464" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O464" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R464" t="n">
-        <v>0.05336427512592412</v>
+        <v>0.07115236683456549</v>
       </c>
       <c r="U464" t="inlineStr">
         <is>
@@ -67432,13 +67432,13 @@
         </is>
       </c>
       <c r="N465" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O465" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R465" t="n">
-        <v>0.03557618341728275</v>
+        <v>0.07115236683456549</v>
       </c>
       <c r="U465" t="inlineStr">
         <is>
@@ -67720,13 +67720,13 @@
         </is>
       </c>
       <c r="N467" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O467" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R467" t="n">
-        <v>0.05336427512592412</v>
+        <v>0.08894045854320688</v>
       </c>
       <c r="U467" t="inlineStr">
         <is>
@@ -67864,13 +67864,13 @@
         </is>
       </c>
       <c r="N468" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="O468" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="R468" t="n">
-        <v>0.4980665678419585</v>
+        <v>0.5514308429678827</v>
       </c>
       <c r="U468" t="inlineStr">
         <is>
@@ -68008,13 +68008,13 @@
         </is>
       </c>
       <c r="N469" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O469" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R469" t="n">
-        <v>0.3023975590469034</v>
+        <v>0.3201856507555447</v>
       </c>
       <c r="U469" t="inlineStr">
         <is>
@@ -68152,13 +68152,13 @@
         </is>
       </c>
       <c r="N470" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="O470" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="R470" t="n">
-        <v>0.5870070263851653</v>
+        <v>0.7470998517629377</v>
       </c>
       <c r="U470" t="inlineStr">
         <is>
@@ -68551,7 +68551,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>41887</v>
+        <v>42093</v>
       </c>
     </row>
     <row r="16">

</xml_diff>